<commit_message>
feat: done parse loai thiet bi
</commit_message>
<xml_diff>
--- a/src/main/resources/qm/public/resources/eQSHImportSchema_vi.xlsx
+++ b/src/main/resources/qm/public/resources/eQSHImportSchema_vi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Qcadoo_demo_clone\mes\mes-plugins\fti-plugins-qm\src\main\resources\qm\public\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42810454-57A1-40F1-BBED-25E8A8690660}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37DF163F-54E6-438E-AB75-D46309EE0457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5235" yWindow="3405" windowWidth="21600" windowHeight="11235" xr2:uid="{1C3DD0E6-ED60-435A-92B4-4D6BBCAE0B6F}"/>
   </bookViews>
@@ -442,7 +442,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B1:B1048576" xr:uid="{F8BEF03A-E2EF-4CFE-86DC-1CB74B159C0A}">
-      <formula1>"01equipment,02internalCalibration,03externalCalibration"</formula1>
+      <formula1>"Thiết bị, Hiệu chuẩn - Trong, Hiệu chuẩn - Ngoài"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>